<commit_message>
jenkins file allure report integration
</commit_message>
<xml_diff>
--- a/test_data/Ram_address.xlsx
+++ b/test_data/Ram_address.xlsx
@@ -86,13 +86,13 @@
     <t>rammyy@1234</t>
   </si>
   <si>
-    <t>Ramm</t>
-  </si>
-  <si>
-    <t>Rannee</t>
-  </si>
-  <si>
-    <t>Yuvjjdd@gmail.com</t>
+    <t>Herrys</t>
+  </si>
+  <si>
+    <t>Herrysf</t>
+  </si>
+  <si>
+    <t>Herrysf@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -137,9 +137,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -421,12 +424,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.77734375" customWidth="1"/>
     <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" customWidth="1"/>
+    <col min="12" max="12" width="11.109375" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" customWidth="1"/>
+    <col min="14" max="14" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -469,7 +479,7 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -514,12 +524,8 @@
         <v>215205</v>
       </c>
       <c r="N2">
-        <v>9858737679</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+        <v>9858537679</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Added new name in file
</commit_message>
<xml_diff>
--- a/test_data/Ram_address.xlsx
+++ b/test_data/Ram_address.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Name</t>
   </si>
@@ -68,9 +68,6 @@
     <t>mobileno</t>
   </si>
   <si>
-    <t>Tiwari</t>
-  </si>
-  <si>
     <t>india</t>
   </si>
   <si>
@@ -86,13 +83,13 @@
     <t>rammyy@1234</t>
   </si>
   <si>
-    <t>Herrys</t>
-  </si>
-  <si>
-    <t>Herrysf</t>
-  </si>
-  <si>
-    <t>Herrysf@gmail.com</t>
+    <t>Jaydev</t>
+  </si>
+  <si>
+    <t>Jaydev@gmail.com</t>
+  </si>
+  <si>
+    <t>Tiwarid</t>
   </si>
 </sst>
 </file>
@@ -485,13 +482,13 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2">
         <v>25</v>
@@ -503,28 +500,28 @@
         <v>1988</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>15</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>16</v>
-      </c>
-      <c r="L2" t="s">
-        <v>17</v>
       </c>
       <c r="M2">
         <v>215205</v>
       </c>
       <c r="N2">
-        <v>9858537679</v>
+        <v>9857537679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>